<commit_message>
Corrected ESD protection wiring and swapped PWRKEY/RESET lines.
</commit_message>
<xml_diff>
--- a/hardware/umay/fabrication/umayBOM.xlsx
+++ b/hardware/umay/fabrication/umayBOM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\recep\OneDrive\Masaüstü\dasProjekt\Git\umay\hardware\umay\Project Outputs for umay\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\recep\OneDrive\Masaüstü\dasProjekt\Git\umay\hardware\umay\fabrication\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4204F3A-C038-437A-A19F-F8D4C1260BE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{686B5F92-3CC5-43C3-A2DC-C0DAC8181FA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -271,9 +271,6 @@
     <t>115I-AEAA</t>
   </si>
   <si>
-    <t>CONN 1x3 Micro Fit 3.00mm</t>
-  </si>
-  <si>
     <t>PJA3404A</t>
   </si>
   <si>
@@ -521,6 +518,9 @@
   </si>
   <si>
     <t>Supplier Unit Price 1</t>
+  </si>
+  <si>
+    <t>L-KLS1-XM1-3.00-1X03-RT</t>
   </si>
 </sst>
 </file>
@@ -531,7 +531,7 @@
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="&quot;₺&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -573,8 +573,13 @@
       <name val="Aptos"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -590,6 +595,24 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF030D42"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -662,7 +685,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -715,9 +738,6 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -762,6 +782,33 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1133,23 +1180,23 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:L98"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="1"/>
-    <col min="2" max="2" width="32.21875" style="16" customWidth="1"/>
-    <col min="3" max="3" width="31.88671875" style="16" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="28.109375" style="16" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="43.6640625" style="16" customWidth="1"/>
-    <col min="6" max="6" width="20.33203125" style="23" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.85546875" style="1"/>
+    <col min="2" max="2" width="32.28515625" style="16" customWidth="1"/>
+    <col min="3" max="3" width="31.85546875" style="16" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="28.140625" style="16" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="43.7109375" style="16" customWidth="1"/>
+    <col min="6" max="6" width="20.28515625" style="22" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="32" style="16" customWidth="1"/>
-    <col min="8" max="8" width="28.33203125" style="23" customWidth="1"/>
-    <col min="9" max="9" width="32.33203125" style="23" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="36.44140625" style="16" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="4.33203125" style="1" customWidth="1"/>
-    <col min="12" max="16384" width="8.88671875" style="1"/>
+    <col min="8" max="8" width="28.28515625" style="22" customWidth="1"/>
+    <col min="9" max="9" width="32.28515625" style="22" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="36.42578125" style="16" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="4.28515625" style="1" customWidth="1"/>
+    <col min="12" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="15"/>
       <c r="C1" s="15"/>
       <c r="D1" s="15"/>
@@ -1160,18 +1207,18 @@
       <c r="I1" s="2"/>
       <c r="J1" s="15"/>
     </row>
-    <row r="2" spans="1:12" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A2" s="3"/>
-      <c r="C2" s="19" t="s">
+      <c r="C2" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="J2" s="29"/>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="J2" s="28"/>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="3"/>
-      <c r="J3" s="30"/>
-    </row>
-    <row r="4" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="J3" s="29"/>
+    </row>
+    <row r="4" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="3"/>
       <c r="B4" s="4"/>
       <c r="C4" s="4" t="s">
@@ -1181,13 +1228,13 @@
         <v>6</v>
       </c>
       <c r="E4" s="4"/>
-      <c r="F4" s="24"/>
+      <c r="F4" s="23"/>
       <c r="G4" s="4"/>
-      <c r="H4" s="24"/>
-      <c r="I4" s="24"/>
-      <c r="J4" s="31"/>
-    </row>
-    <row r="5" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="H4" s="23"/>
+      <c r="I4" s="23"/>
+      <c r="J4" s="30"/>
+    </row>
+    <row r="5" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>
       <c r="B5" s="4"/>
       <c r="C5" s="4" t="s">
@@ -1197,13 +1244,13 @@
         <v>6</v>
       </c>
       <c r="E5" s="4"/>
-      <c r="F5" s="24"/>
+      <c r="F5" s="23"/>
       <c r="G5" s="4"/>
-      <c r="H5" s="24"/>
-      <c r="I5" s="24"/>
-      <c r="J5" s="31"/>
-    </row>
-    <row r="6" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="H5" s="23"/>
+      <c r="I5" s="23"/>
+      <c r="J5" s="30"/>
+    </row>
+    <row r="6" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="3"/>
       <c r="B6" s="4"/>
       <c r="C6" s="4" t="s">
@@ -1213,13 +1260,13 @@
         <v>7</v>
       </c>
       <c r="E6" s="4"/>
-      <c r="F6" s="24"/>
+      <c r="F6" s="23"/>
       <c r="G6" s="4"/>
-      <c r="H6" s="24"/>
-      <c r="I6" s="24"/>
-      <c r="J6" s="31"/>
-    </row>
-    <row r="7" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="H6" s="23"/>
+      <c r="I6" s="23"/>
+      <c r="J6" s="30"/>
+    </row>
+    <row r="7" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="3"/>
       <c r="B7" s="4"/>
       <c r="C7" s="4" t="s">
@@ -1229,49 +1276,49 @@
         <v>8</v>
       </c>
       <c r="E7" s="4"/>
-      <c r="F7" s="24"/>
+      <c r="F7" s="23"/>
       <c r="G7" s="4"/>
-      <c r="H7" s="24"/>
-      <c r="I7" s="24"/>
-      <c r="J7" s="31"/>
-    </row>
-    <row r="8" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="H7" s="23"/>
+      <c r="I7" s="23"/>
+      <c r="J7" s="30"/>
+    </row>
+    <row r="8" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="3"/>
       <c r="B8" s="4"/>
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
       <c r="E8" s="4"/>
-      <c r="F8" s="24"/>
+      <c r="F8" s="23"/>
       <c r="G8" s="4"/>
-      <c r="H8" s="24"/>
-      <c r="I8" s="24"/>
-      <c r="J8" s="31"/>
-    </row>
-    <row r="9" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="H8" s="23"/>
+      <c r="I8" s="23"/>
+      <c r="J8" s="30"/>
+    </row>
+    <row r="9" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9" s="3"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
       <c r="E9" s="4"/>
-      <c r="F9" s="24"/>
+      <c r="F9" s="23"/>
       <c r="G9" s="4"/>
-      <c r="H9" s="24"/>
-      <c r="I9" s="24"/>
-      <c r="J9" s="31"/>
-    </row>
-    <row r="10" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H9" s="23"/>
+      <c r="I9" s="23"/>
+      <c r="J9" s="30"/>
+    </row>
+    <row r="10" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
       <c r="E10" s="4"/>
-      <c r="F10" s="24"/>
+      <c r="F10" s="23"/>
       <c r="G10" s="4"/>
-      <c r="H10" s="24"/>
-      <c r="I10" s="24"/>
-      <c r="J10" s="32"/>
-    </row>
-    <row r="11" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="H10" s="23"/>
+      <c r="I10" s="23"/>
+      <c r="J10" s="31"/>
+    </row>
+    <row r="11" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B11" s="6" t="s">
         <v>9</v>
       </c>
@@ -1279,40 +1326,40 @@
         <v>57</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F11" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="G11" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="G11" s="6" t="s">
+      <c r="H11" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="H11" s="6" t="s">
+      <c r="I11" s="6" t="s">
         <v>160</v>
-      </c>
-      <c r="I11" s="6" t="s">
-        <v>161</v>
       </c>
       <c r="J11" s="6" t="s">
         <v>5</v>
       </c>
       <c r="L11" s="7"/>
     </row>
-    <row r="12" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B12" s="17" t="s">
+    <row r="12" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B12" s="33" t="s">
         <v>10</v>
       </c>
-      <c r="C12" s="17" t="s">
+      <c r="C12" s="33" t="s">
         <v>58</v>
       </c>
-      <c r="D12" s="17" t="s">
-        <v>105</v>
-      </c>
-      <c r="E12" s="17" t="s">
-        <v>128</v>
+      <c r="D12" s="33" t="s">
+        <v>104</v>
+      </c>
+      <c r="E12" s="33" t="s">
+        <v>127</v>
       </c>
       <c r="F12" s="8">
         <v>2</v>
@@ -1323,40 +1370,40 @@
       <c r="J12" s="17"/>
       <c r="L12" s="10"/>
     </row>
-    <row r="13" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B13" s="18" t="s">
+    <row r="13" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B13" s="33" t="s">
         <v>11</v>
       </c>
-      <c r="C13" s="20" t="s">
+      <c r="C13" s="34" t="s">
         <v>59</v>
       </c>
-      <c r="D13" s="20" t="s">
-        <v>106</v>
-      </c>
-      <c r="E13" s="20" t="s">
-        <v>129</v>
+      <c r="D13" s="34" t="s">
+        <v>105</v>
+      </c>
+      <c r="E13" s="34" t="s">
+        <v>128</v>
       </c>
       <c r="F13" s="11">
         <v>17</v>
       </c>
-      <c r="G13" s="20"/>
+      <c r="G13" s="19"/>
       <c r="H13" s="12"/>
       <c r="I13" s="13"/>
-      <c r="J13" s="33"/>
+      <c r="J13" s="32"/>
       <c r="L13" s="10"/>
     </row>
-    <row r="14" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B14" s="17" t="s">
+    <row r="14" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B14" s="33" t="s">
         <v>12</v>
       </c>
-      <c r="C14" s="17" t="s">
+      <c r="C14" s="33" t="s">
         <v>60</v>
       </c>
-      <c r="D14" s="17" t="s">
-        <v>105</v>
-      </c>
-      <c r="E14" s="17" t="s">
-        <v>128</v>
+      <c r="D14" s="33" t="s">
+        <v>104</v>
+      </c>
+      <c r="E14" s="33" t="s">
+        <v>127</v>
       </c>
       <c r="F14" s="8">
         <v>5</v>
@@ -1367,40 +1414,40 @@
       <c r="J14" s="17"/>
       <c r="L14" s="10"/>
     </row>
-    <row r="15" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B15" s="18" t="s">
+    <row r="15" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B15" s="33" t="s">
         <v>13</v>
       </c>
-      <c r="C15" s="20" t="s">
+      <c r="C15" s="34" t="s">
         <v>61</v>
       </c>
-      <c r="D15" s="20" t="s">
-        <v>106</v>
-      </c>
-      <c r="E15" s="20" t="s">
-        <v>129</v>
+      <c r="D15" s="34" t="s">
+        <v>105</v>
+      </c>
+      <c r="E15" s="34" t="s">
+        <v>128</v>
       </c>
       <c r="F15" s="11">
         <v>2</v>
       </c>
-      <c r="G15" s="20"/>
+      <c r="G15" s="19"/>
       <c r="H15" s="12"/>
       <c r="I15" s="13"/>
-      <c r="J15" s="33"/>
+      <c r="J15" s="32"/>
       <c r="L15" s="10"/>
     </row>
-    <row r="16" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B16" s="17" t="s">
+    <row r="16" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B16" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="C16" s="17" t="s">
+      <c r="C16" s="33" t="s">
         <v>62</v>
       </c>
-      <c r="D16" s="17" t="s">
-        <v>106</v>
-      </c>
-      <c r="E16" s="17" t="s">
-        <v>129</v>
+      <c r="D16" s="33" t="s">
+        <v>105</v>
+      </c>
+      <c r="E16" s="33" t="s">
+        <v>128</v>
       </c>
       <c r="F16" s="8">
         <v>2</v>
@@ -1411,40 +1458,40 @@
       <c r="J16" s="17"/>
       <c r="L16" s="10"/>
     </row>
-    <row r="17" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B17" s="18" t="s">
+    <row r="17" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B17" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="C17" s="20" t="s">
+      <c r="C17" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="D17" s="20" t="s">
-        <v>105</v>
-      </c>
-      <c r="E17" s="20" t="s">
-        <v>128</v>
+      <c r="D17" s="34" t="s">
+        <v>104</v>
+      </c>
+      <c r="E17" s="34" t="s">
+        <v>127</v>
       </c>
       <c r="F17" s="11">
         <v>1</v>
       </c>
-      <c r="G17" s="20"/>
+      <c r="G17" s="19"/>
       <c r="H17" s="12"/>
       <c r="I17" s="13"/>
-      <c r="J17" s="33"/>
+      <c r="J17" s="32"/>
       <c r="L17" s="10"/>
     </row>
-    <row r="18" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B18" s="17" t="s">
+    <row r="18" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B18" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="C18" s="17" t="s">
+      <c r="C18" s="33" t="s">
         <v>64</v>
       </c>
-      <c r="D18" s="17" t="s">
-        <v>107</v>
-      </c>
-      <c r="E18" s="17" t="s">
-        <v>130</v>
+      <c r="D18" s="33" t="s">
+        <v>106</v>
+      </c>
+      <c r="E18" s="33" t="s">
+        <v>129</v>
       </c>
       <c r="F18" s="8">
         <v>2</v>
@@ -1455,40 +1502,40 @@
       <c r="J18" s="17"/>
       <c r="L18" s="10"/>
     </row>
-    <row r="19" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B19" s="18" t="s">
+    <row r="19" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B19" s="33" t="s">
         <v>17</v>
       </c>
-      <c r="C19" s="20" t="s">
+      <c r="C19" s="34" t="s">
         <v>65</v>
       </c>
-      <c r="D19" s="20" t="s">
-        <v>106</v>
-      </c>
-      <c r="E19" s="20" t="s">
-        <v>129</v>
+      <c r="D19" s="34" t="s">
+        <v>105</v>
+      </c>
+      <c r="E19" s="34" t="s">
+        <v>128</v>
       </c>
       <c r="F19" s="11">
         <v>2</v>
       </c>
-      <c r="G19" s="20"/>
+      <c r="G19" s="19"/>
       <c r="H19" s="12"/>
       <c r="I19" s="13"/>
-      <c r="J19" s="33"/>
+      <c r="J19" s="32"/>
       <c r="L19" s="10"/>
     </row>
-    <row r="20" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B20" s="17" t="s">
+    <row r="20" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B20" s="33" t="s">
         <v>18</v>
       </c>
-      <c r="C20" s="17" t="s">
+      <c r="C20" s="33" t="s">
         <v>66</v>
       </c>
-      <c r="D20" s="17" t="s">
-        <v>106</v>
-      </c>
-      <c r="E20" s="17" t="s">
-        <v>129</v>
+      <c r="D20" s="33" t="s">
+        <v>105</v>
+      </c>
+      <c r="E20" s="33" t="s">
+        <v>128</v>
       </c>
       <c r="F20" s="8">
         <v>5</v>
@@ -1499,40 +1546,40 @@
       <c r="J20" s="17"/>
       <c r="L20" s="10"/>
     </row>
-    <row r="21" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B21" s="18" t="s">
+    <row r="21" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B21" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="C21" s="20" t="s">
+      <c r="C21" s="34" t="s">
         <v>67</v>
       </c>
-      <c r="D21" s="20" t="s">
-        <v>106</v>
-      </c>
-      <c r="E21" s="20" t="s">
-        <v>129</v>
+      <c r="D21" s="34" t="s">
+        <v>105</v>
+      </c>
+      <c r="E21" s="34" t="s">
+        <v>128</v>
       </c>
       <c r="F21" s="11">
         <v>2</v>
       </c>
-      <c r="G21" s="20"/>
+      <c r="G21" s="19"/>
       <c r="H21" s="12"/>
       <c r="I21" s="13"/>
-      <c r="J21" s="33"/>
+      <c r="J21" s="32"/>
       <c r="L21" s="10"/>
     </row>
-    <row r="22" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B22" s="17" t="s">
+    <row r="22" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B22" s="33" t="s">
         <v>20</v>
       </c>
-      <c r="C22" s="17" t="s">
+      <c r="C22" s="33" t="s">
         <v>68</v>
       </c>
-      <c r="D22" s="17" t="s">
-        <v>106</v>
-      </c>
-      <c r="E22" s="17" t="s">
-        <v>129</v>
+      <c r="D22" s="33" t="s">
+        <v>105</v>
+      </c>
+      <c r="E22" s="33" t="s">
+        <v>128</v>
       </c>
       <c r="F22" s="8">
         <v>2</v>
@@ -1543,40 +1590,40 @@
       <c r="J22" s="17"/>
       <c r="L22" s="10"/>
     </row>
-    <row r="23" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B23" s="18" t="s">
+    <row r="23" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B23" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="C23" s="20" t="s">
+      <c r="C23" s="34" t="s">
         <v>69</v>
       </c>
-      <c r="D23" s="20" t="s">
+      <c r="D23" s="34" t="s">
         <v>69</v>
       </c>
-      <c r="E23" s="20" t="s">
-        <v>131</v>
+      <c r="E23" s="34" t="s">
+        <v>130</v>
       </c>
       <c r="F23" s="11">
         <v>2</v>
       </c>
-      <c r="G23" s="20"/>
+      <c r="G23" s="19"/>
       <c r="H23" s="12"/>
       <c r="I23" s="13"/>
-      <c r="J23" s="33"/>
+      <c r="J23" s="32"/>
       <c r="L23" s="10"/>
     </row>
-    <row r="24" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B24" s="17" t="s">
+    <row r="24" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B24" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="C24" s="17" t="s">
+      <c r="C24" s="33" t="s">
         <v>70</v>
       </c>
-      <c r="D24" s="17" t="s">
-        <v>108</v>
-      </c>
-      <c r="E24" s="17" t="s">
-        <v>132</v>
+      <c r="D24" s="33" t="s">
+        <v>107</v>
+      </c>
+      <c r="E24" s="33" t="s">
+        <v>131</v>
       </c>
       <c r="F24" s="8">
         <v>1</v>
@@ -1587,40 +1634,40 @@
       <c r="J24" s="17"/>
       <c r="L24" s="10"/>
     </row>
-    <row r="25" spans="2:12" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="B25" s="18" t="s">
+    <row r="25" spans="2:12" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="B25" s="35" t="s">
         <v>23</v>
       </c>
-      <c r="C25" s="20" t="s">
+      <c r="C25" s="36" t="s">
         <v>71</v>
       </c>
-      <c r="D25" s="20" t="s">
-        <v>109</v>
-      </c>
-      <c r="E25" s="20" t="s">
-        <v>133</v>
-      </c>
-      <c r="F25" s="11">
+      <c r="D25" s="36" t="s">
+        <v>108</v>
+      </c>
+      <c r="E25" s="36" t="s">
+        <v>132</v>
+      </c>
+      <c r="F25" s="38">
         <v>1</v>
       </c>
-      <c r="G25" s="20"/>
+      <c r="G25" s="19"/>
       <c r="H25" s="12"/>
       <c r="I25" s="13"/>
-      <c r="J25" s="33"/>
+      <c r="J25" s="32"/>
       <c r="L25" s="10"/>
     </row>
-    <row r="26" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B26" s="17" t="s">
+    <row r="26" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B26" s="33" t="s">
         <v>24</v>
       </c>
-      <c r="C26" s="17" t="s">
+      <c r="C26" s="33" t="s">
         <v>72</v>
       </c>
-      <c r="D26" s="17" t="s">
-        <v>110</v>
-      </c>
-      <c r="E26" s="17" t="s">
-        <v>134</v>
+      <c r="D26" s="33" t="s">
+        <v>109</v>
+      </c>
+      <c r="E26" s="33" t="s">
+        <v>133</v>
       </c>
       <c r="F26" s="8">
         <v>1</v>
@@ -1631,40 +1678,40 @@
       <c r="J26" s="17"/>
       <c r="L26" s="10"/>
     </row>
-    <row r="27" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B27" s="18" t="s">
+    <row r="27" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B27" s="33" t="s">
         <v>25</v>
       </c>
-      <c r="C27" s="20" t="s">
+      <c r="C27" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="D27" s="20" t="s">
-        <v>111</v>
-      </c>
-      <c r="E27" s="20" t="s">
-        <v>135</v>
+      <c r="D27" s="34" t="s">
+        <v>110</v>
+      </c>
+      <c r="E27" s="34" t="s">
+        <v>134</v>
       </c>
       <c r="F27" s="11">
         <v>1</v>
       </c>
-      <c r="G27" s="20"/>
+      <c r="G27" s="19"/>
       <c r="H27" s="12"/>
       <c r="I27" s="13"/>
-      <c r="J27" s="33"/>
+      <c r="J27" s="32"/>
       <c r="L27" s="10"/>
     </row>
-    <row r="28" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B28" s="17" t="s">
+    <row r="28" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B28" s="37" t="s">
         <v>26</v>
       </c>
-      <c r="C28" s="17" t="s">
+      <c r="C28" s="37" t="s">
         <v>74</v>
       </c>
-      <c r="D28" s="17" t="s">
-        <v>112</v>
-      </c>
-      <c r="E28" s="17" t="s">
-        <v>136</v>
+      <c r="D28" s="37" t="s">
+        <v>111</v>
+      </c>
+      <c r="E28" s="37" t="s">
+        <v>135</v>
       </c>
       <c r="F28" s="8">
         <v>1</v>
@@ -1675,40 +1722,40 @@
       <c r="J28" s="17"/>
       <c r="L28" s="10"/>
     </row>
-    <row r="29" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B29" s="18" t="s">
+    <row r="29" spans="2:12" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B29" s="33" t="s">
         <v>27</v>
       </c>
-      <c r="C29" s="20" t="s">
+      <c r="C29" s="34" t="s">
         <v>75</v>
       </c>
-      <c r="D29" s="20" t="s">
-        <v>113</v>
-      </c>
-      <c r="E29" s="20" t="s">
-        <v>137</v>
+      <c r="D29" s="34" t="s">
+        <v>112</v>
+      </c>
+      <c r="E29" s="34" t="s">
+        <v>136</v>
       </c>
       <c r="F29" s="11">
         <v>1</v>
       </c>
-      <c r="G29" s="20"/>
+      <c r="G29" s="19"/>
       <c r="H29" s="12"/>
       <c r="I29" s="13"/>
-      <c r="J29" s="33"/>
+      <c r="J29" s="32"/>
       <c r="L29" s="10"/>
     </row>
-    <row r="30" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B30" s="17" t="s">
+    <row r="30" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B30" s="33" t="s">
         <v>28</v>
       </c>
-      <c r="C30" s="17" t="s">
+      <c r="C30" s="33" t="s">
         <v>76</v>
       </c>
-      <c r="D30" s="17" t="s">
-        <v>114</v>
-      </c>
-      <c r="E30" s="17" t="s">
-        <v>138</v>
+      <c r="D30" s="33" t="s">
+        <v>113</v>
+      </c>
+      <c r="E30" s="33" t="s">
+        <v>137</v>
       </c>
       <c r="F30" s="8">
         <v>1</v>
@@ -1719,42 +1766,42 @@
       <c r="J30" s="17"/>
       <c r="L30" s="10"/>
     </row>
-    <row r="31" spans="2:12" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B31" s="18" t="s">
+    <row r="31" spans="2:12" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B31" s="33" t="s">
         <v>29</v>
       </c>
-      <c r="C31" s="20" t="s">
+      <c r="C31" s="34" t="s">
         <v>77</v>
       </c>
-      <c r="D31" s="20" t="s">
+      <c r="D31" s="34" t="s">
         <v>77</v>
       </c>
-      <c r="E31" s="20" t="s">
-        <v>139</v>
+      <c r="E31" s="34" t="s">
+        <v>138</v>
       </c>
       <c r="F31" s="11">
         <v>1</v>
       </c>
-      <c r="G31" s="20"/>
+      <c r="G31" s="19"/>
       <c r="H31" s="12"/>
       <c r="I31" s="13"/>
-      <c r="J31" s="33"/>
+      <c r="J31" s="32"/>
       <c r="L31" s="10"/>
     </row>
-    <row r="32" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B32" s="17" t="s">
+    <row r="32" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B32" s="33" t="s">
         <v>30</v>
       </c>
-      <c r="C32" s="17" t="s">
-        <v>78</v>
-      </c>
-      <c r="D32" s="17" t="s">
-        <v>115</v>
-      </c>
-      <c r="E32" s="17" t="s">
-        <v>140</v>
-      </c>
-      <c r="F32" s="8">
+      <c r="C32" s="33" t="s">
+        <v>161</v>
+      </c>
+      <c r="D32" s="33" t="s">
+        <v>114</v>
+      </c>
+      <c r="E32" s="33" t="s">
+        <v>139</v>
+      </c>
+      <c r="F32" s="39">
         <v>1</v>
       </c>
       <c r="G32" s="17"/>
@@ -1763,40 +1810,40 @@
       <c r="J32" s="17"/>
       <c r="L32" s="10"/>
     </row>
-    <row r="33" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B33" s="18" t="s">
+    <row r="33" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B33" s="33" t="s">
         <v>31</v>
       </c>
-      <c r="C33" s="20" t="s">
-        <v>79</v>
-      </c>
-      <c r="D33" s="20" t="s">
-        <v>116</v>
-      </c>
-      <c r="E33" s="20" t="s">
-        <v>141</v>
+      <c r="C33" s="34" t="s">
+        <v>78</v>
+      </c>
+      <c r="D33" s="34" t="s">
+        <v>115</v>
+      </c>
+      <c r="E33" s="34" t="s">
+        <v>140</v>
       </c>
       <c r="F33" s="11">
         <v>4</v>
       </c>
-      <c r="G33" s="20"/>
+      <c r="G33" s="19"/>
       <c r="H33" s="12"/>
       <c r="I33" s="13"/>
-      <c r="J33" s="33"/>
+      <c r="J33" s="32"/>
       <c r="L33" s="10"/>
     </row>
-    <row r="34" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B34" s="17" t="s">
+    <row r="34" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B34" s="33" t="s">
         <v>32</v>
       </c>
-      <c r="C34" s="17" t="s">
-        <v>80</v>
-      </c>
-      <c r="D34" s="17" t="s">
-        <v>116</v>
-      </c>
-      <c r="E34" s="17" t="s">
-        <v>142</v>
+      <c r="C34" s="33" t="s">
+        <v>79</v>
+      </c>
+      <c r="D34" s="33" t="s">
+        <v>115</v>
+      </c>
+      <c r="E34" s="33" t="s">
+        <v>141</v>
       </c>
       <c r="F34" s="8">
         <v>2</v>
@@ -1807,40 +1854,40 @@
       <c r="J34" s="17"/>
       <c r="L34" s="10"/>
     </row>
-    <row r="35" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B35" s="18" t="s">
+    <row r="35" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B35" s="33" t="s">
         <v>33</v>
       </c>
-      <c r="C35" s="20" t="s">
-        <v>81</v>
-      </c>
-      <c r="D35" s="20" t="s">
-        <v>117</v>
-      </c>
-      <c r="E35" s="20" t="s">
-        <v>143</v>
-      </c>
-      <c r="F35" s="11">
+      <c r="C35" s="34" t="s">
+        <v>80</v>
+      </c>
+      <c r="D35" s="34" t="s">
+        <v>116</v>
+      </c>
+      <c r="E35" s="34" t="s">
+        <v>142</v>
+      </c>
+      <c r="F35" s="38">
         <v>3</v>
       </c>
-      <c r="G35" s="20"/>
+      <c r="G35" s="19"/>
       <c r="H35" s="12"/>
       <c r="I35" s="13"/>
-      <c r="J35" s="33"/>
+      <c r="J35" s="32"/>
       <c r="L35" s="10"/>
     </row>
-    <row r="36" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B36" s="17" t="s">
+    <row r="36" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B36" s="33" t="s">
         <v>34</v>
       </c>
-      <c r="C36" s="17" t="s">
-        <v>82</v>
-      </c>
-      <c r="D36" s="17" t="s">
-        <v>117</v>
-      </c>
-      <c r="E36" s="17" t="s">
-        <v>143</v>
+      <c r="C36" s="33" t="s">
+        <v>81</v>
+      </c>
+      <c r="D36" s="33" t="s">
+        <v>116</v>
+      </c>
+      <c r="E36" s="33" t="s">
+        <v>142</v>
       </c>
       <c r="F36" s="8">
         <v>9</v>
@@ -1851,40 +1898,40 @@
       <c r="J36" s="17"/>
       <c r="L36" s="10"/>
     </row>
-    <row r="37" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B37" s="18" t="s">
+    <row r="37" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B37" s="33" t="s">
         <v>35</v>
       </c>
-      <c r="C37" s="20" t="s">
-        <v>83</v>
-      </c>
-      <c r="D37" s="20" t="s">
-        <v>117</v>
-      </c>
-      <c r="E37" s="20" t="s">
-        <v>143</v>
+      <c r="C37" s="34" t="s">
+        <v>82</v>
+      </c>
+      <c r="D37" s="34" t="s">
+        <v>116</v>
+      </c>
+      <c r="E37" s="34" t="s">
+        <v>142</v>
       </c>
       <c r="F37" s="11">
         <v>2</v>
       </c>
-      <c r="G37" s="20"/>
+      <c r="G37" s="19"/>
       <c r="H37" s="12"/>
       <c r="I37" s="13"/>
-      <c r="J37" s="33"/>
+      <c r="J37" s="32"/>
       <c r="L37" s="10"/>
     </row>
-    <row r="38" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B38" s="17" t="s">
+    <row r="38" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B38" s="33" t="s">
         <v>36</v>
       </c>
-      <c r="C38" s="17" t="s">
-        <v>84</v>
-      </c>
-      <c r="D38" s="17" t="s">
-        <v>117</v>
-      </c>
-      <c r="E38" s="17" t="s">
-        <v>143</v>
+      <c r="C38" s="33" t="s">
+        <v>83</v>
+      </c>
+      <c r="D38" s="33" t="s">
+        <v>116</v>
+      </c>
+      <c r="E38" s="33" t="s">
+        <v>142</v>
       </c>
       <c r="F38" s="8">
         <v>4</v>
@@ -1895,40 +1942,40 @@
       <c r="J38" s="17"/>
       <c r="L38" s="10"/>
     </row>
-    <row r="39" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B39" s="18" t="s">
+    <row r="39" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B39" s="33" t="s">
         <v>37</v>
       </c>
-      <c r="C39" s="20" t="s">
-        <v>85</v>
-      </c>
-      <c r="D39" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="E39" s="20" t="s">
-        <v>144</v>
+      <c r="C39" s="34" t="s">
+        <v>84</v>
+      </c>
+      <c r="D39" s="34" t="s">
+        <v>117</v>
+      </c>
+      <c r="E39" s="34" t="s">
+        <v>143</v>
       </c>
       <c r="F39" s="11">
         <v>2</v>
       </c>
-      <c r="G39" s="20"/>
+      <c r="G39" s="19"/>
       <c r="H39" s="12"/>
       <c r="I39" s="13"/>
-      <c r="J39" s="33"/>
+      <c r="J39" s="32"/>
       <c r="L39" s="10"/>
     </row>
-    <row r="40" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B40" s="17" t="s">
+    <row r="40" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B40" s="33" t="s">
         <v>38</v>
       </c>
-      <c r="C40" s="17" t="s">
-        <v>85</v>
-      </c>
-      <c r="D40" s="17" t="s">
-        <v>117</v>
-      </c>
-      <c r="E40" s="17" t="s">
-        <v>143</v>
+      <c r="C40" s="33" t="s">
+        <v>84</v>
+      </c>
+      <c r="D40" s="33" t="s">
+        <v>116</v>
+      </c>
+      <c r="E40" s="33" t="s">
+        <v>142</v>
       </c>
       <c r="F40" s="8">
         <v>4</v>
@@ -1939,40 +1986,40 @@
       <c r="J40" s="17"/>
       <c r="L40" s="10"/>
     </row>
-    <row r="41" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B41" s="18" t="s">
+    <row r="41" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B41" s="33" t="s">
         <v>39</v>
       </c>
-      <c r="C41" s="20" t="s">
-        <v>86</v>
-      </c>
-      <c r="D41" s="20" t="s">
-        <v>117</v>
-      </c>
-      <c r="E41" s="20" t="s">
-        <v>143</v>
+      <c r="C41" s="34" t="s">
+        <v>85</v>
+      </c>
+      <c r="D41" s="34" t="s">
+        <v>116</v>
+      </c>
+      <c r="E41" s="34" t="s">
+        <v>142</v>
       </c>
       <c r="F41" s="11">
         <v>1</v>
       </c>
-      <c r="G41" s="20"/>
+      <c r="G41" s="19"/>
       <c r="H41" s="12"/>
       <c r="I41" s="13"/>
-      <c r="J41" s="33"/>
+      <c r="J41" s="32"/>
       <c r="L41" s="10"/>
     </row>
-    <row r="42" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B42" s="17" t="s">
+    <row r="42" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B42" s="33" t="s">
         <v>40</v>
       </c>
-      <c r="C42" s="17" t="s">
-        <v>87</v>
-      </c>
-      <c r="D42" s="17" t="s">
-        <v>117</v>
-      </c>
-      <c r="E42" s="17" t="s">
-        <v>143</v>
+      <c r="C42" s="33" t="s">
+        <v>86</v>
+      </c>
+      <c r="D42" s="33" t="s">
+        <v>116</v>
+      </c>
+      <c r="E42" s="33" t="s">
+        <v>142</v>
       </c>
       <c r="F42" s="8">
         <v>1</v>
@@ -1983,40 +2030,40 @@
       <c r="J42" s="17"/>
       <c r="L42" s="10"/>
     </row>
-    <row r="43" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B43" s="18" t="s">
+    <row r="43" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B43" s="33" t="s">
         <v>41</v>
       </c>
-      <c r="C43" s="20" t="s">
-        <v>88</v>
-      </c>
-      <c r="D43" s="20" t="s">
-        <v>117</v>
-      </c>
-      <c r="E43" s="20" t="s">
-        <v>143</v>
+      <c r="C43" s="34" t="s">
+        <v>87</v>
+      </c>
+      <c r="D43" s="34" t="s">
+        <v>116</v>
+      </c>
+      <c r="E43" s="34" t="s">
+        <v>142</v>
       </c>
       <c r="F43" s="11">
         <v>2</v>
       </c>
-      <c r="G43" s="20"/>
+      <c r="G43" s="19"/>
       <c r="H43" s="12"/>
       <c r="I43" s="13"/>
-      <c r="J43" s="33"/>
+      <c r="J43" s="32"/>
       <c r="L43" s="10"/>
     </row>
-    <row r="44" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B44" s="17" t="s">
+    <row r="44" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B44" s="33" t="s">
         <v>42</v>
       </c>
-      <c r="C44" s="17" t="s">
-        <v>89</v>
-      </c>
-      <c r="D44" s="17" t="s">
-        <v>117</v>
-      </c>
-      <c r="E44" s="17" t="s">
-        <v>143</v>
+      <c r="C44" s="33" t="s">
+        <v>88</v>
+      </c>
+      <c r="D44" s="33" t="s">
+        <v>116</v>
+      </c>
+      <c r="E44" s="33" t="s">
+        <v>142</v>
       </c>
       <c r="F44" s="8">
         <v>1</v>
@@ -2027,42 +2074,42 @@
       <c r="J44" s="17"/>
       <c r="L44" s="10"/>
     </row>
-    <row r="45" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B45" s="18" t="s">
+    <row r="45" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B45" s="33" t="s">
         <v>43</v>
       </c>
-      <c r="C45" s="20" t="s">
-        <v>90</v>
-      </c>
-      <c r="D45" s="20" t="s">
-        <v>117</v>
-      </c>
-      <c r="E45" s="20" t="s">
-        <v>143</v>
+      <c r="C45" s="34" t="s">
+        <v>89</v>
+      </c>
+      <c r="D45" s="34" t="s">
+        <v>116</v>
+      </c>
+      <c r="E45" s="34" t="s">
+        <v>142</v>
       </c>
       <c r="F45" s="11">
         <v>2</v>
       </c>
-      <c r="G45" s="20"/>
+      <c r="G45" s="19"/>
       <c r="H45" s="12"/>
       <c r="I45" s="13"/>
-      <c r="J45" s="33"/>
+      <c r="J45" s="32"/>
       <c r="L45" s="10"/>
     </row>
-    <row r="46" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B46" s="17" t="s">
+    <row r="46" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B46" s="33" t="s">
         <v>44</v>
       </c>
-      <c r="C46" s="17" t="s">
-        <v>91</v>
-      </c>
-      <c r="D46" s="17" t="s">
-        <v>119</v>
-      </c>
-      <c r="E46" s="17" t="s">
-        <v>145</v>
-      </c>
-      <c r="F46" s="8">
+      <c r="C46" s="33" t="s">
+        <v>90</v>
+      </c>
+      <c r="D46" s="33" t="s">
+        <v>118</v>
+      </c>
+      <c r="E46" s="33" t="s">
+        <v>144</v>
+      </c>
+      <c r="F46" s="39">
         <v>1</v>
       </c>
       <c r="G46" s="17"/>
@@ -2071,40 +2118,40 @@
       <c r="J46" s="17"/>
       <c r="L46" s="10"/>
     </row>
-    <row r="47" spans="2:12" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="B47" s="18" t="s">
+    <row r="47" spans="2:12" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="B47" s="33" t="s">
         <v>45</v>
       </c>
-      <c r="C47" s="20" t="s">
-        <v>92</v>
-      </c>
-      <c r="D47" s="20" t="s">
-        <v>92</v>
-      </c>
-      <c r="E47" s="20" t="s">
-        <v>146</v>
+      <c r="C47" s="34" t="s">
+        <v>91</v>
+      </c>
+      <c r="D47" s="34" t="s">
+        <v>91</v>
+      </c>
+      <c r="E47" s="34" t="s">
+        <v>145</v>
       </c>
       <c r="F47" s="11">
         <v>1</v>
       </c>
-      <c r="G47" s="20"/>
+      <c r="G47" s="19"/>
       <c r="H47" s="12"/>
       <c r="I47" s="13"/>
-      <c r="J47" s="33"/>
+      <c r="J47" s="32"/>
       <c r="L47" s="10"/>
     </row>
-    <row r="48" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B48" s="17" t="s">
+    <row r="48" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B48" s="33" t="s">
         <v>46</v>
       </c>
-      <c r="C48" s="17" t="s">
-        <v>93</v>
-      </c>
-      <c r="D48" s="17" t="s">
-        <v>93</v>
-      </c>
-      <c r="E48" s="17" t="s">
-        <v>147</v>
+      <c r="C48" s="33" t="s">
+        <v>92</v>
+      </c>
+      <c r="D48" s="33" t="s">
+        <v>92</v>
+      </c>
+      <c r="E48" s="33" t="s">
+        <v>146</v>
       </c>
       <c r="F48" s="8">
         <v>6</v>
@@ -2115,40 +2162,40 @@
       <c r="J48" s="17"/>
       <c r="L48" s="10"/>
     </row>
-    <row r="49" spans="2:12" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="B49" s="18" t="s">
+    <row r="49" spans="2:12" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="B49" s="40" t="s">
         <v>47</v>
       </c>
-      <c r="C49" s="20" t="s">
-        <v>94</v>
-      </c>
-      <c r="D49" s="20" t="s">
-        <v>120</v>
-      </c>
-      <c r="E49" s="20" t="s">
-        <v>148</v>
+      <c r="C49" s="41" t="s">
+        <v>93</v>
+      </c>
+      <c r="D49" s="41" t="s">
+        <v>119</v>
+      </c>
+      <c r="E49" s="41" t="s">
+        <v>147</v>
       </c>
       <c r="F49" s="11">
         <v>1</v>
       </c>
-      <c r="G49" s="20"/>
+      <c r="G49" s="19"/>
       <c r="H49" s="12"/>
       <c r="I49" s="13"/>
-      <c r="J49" s="33"/>
+      <c r="J49" s="32"/>
       <c r="L49" s="10"/>
     </row>
-    <row r="50" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B50" s="17" t="s">
+    <row r="50" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B50" s="33" t="s">
         <v>48</v>
       </c>
-      <c r="C50" s="17" t="s">
-        <v>95</v>
-      </c>
-      <c r="D50" s="17" t="s">
-        <v>95</v>
-      </c>
-      <c r="E50" s="17" t="s">
-        <v>149</v>
+      <c r="C50" s="33" t="s">
+        <v>94</v>
+      </c>
+      <c r="D50" s="33" t="s">
+        <v>94</v>
+      </c>
+      <c r="E50" s="33" t="s">
+        <v>148</v>
       </c>
       <c r="F50" s="8">
         <v>1</v>
@@ -2159,40 +2206,40 @@
       <c r="J50" s="17"/>
       <c r="L50" s="10"/>
     </row>
-    <row r="51" spans="2:12" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B51" s="18" t="s">
+    <row r="51" spans="2:12" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B51" s="33" t="s">
         <v>49</v>
       </c>
-      <c r="C51" s="20" t="s">
-        <v>96</v>
-      </c>
-      <c r="D51" s="20" t="s">
-        <v>96</v>
-      </c>
-      <c r="E51" s="20" t="s">
-        <v>150</v>
+      <c r="C51" s="34" t="s">
+        <v>95</v>
+      </c>
+      <c r="D51" s="34" t="s">
+        <v>95</v>
+      </c>
+      <c r="E51" s="34" t="s">
+        <v>149</v>
       </c>
       <c r="F51" s="11">
         <v>1</v>
       </c>
-      <c r="G51" s="20"/>
+      <c r="G51" s="19"/>
       <c r="H51" s="12"/>
       <c r="I51" s="13"/>
-      <c r="J51" s="33"/>
+      <c r="J51" s="32"/>
       <c r="L51" s="10"/>
     </row>
-    <row r="52" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B52" s="17" t="s">
+    <row r="52" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B52" s="33" t="s">
         <v>50</v>
       </c>
-      <c r="C52" s="17" t="s">
-        <v>97</v>
-      </c>
-      <c r="D52" s="17" t="s">
-        <v>97</v>
-      </c>
-      <c r="E52" s="17" t="s">
-        <v>151</v>
+      <c r="C52" s="33" t="s">
+        <v>96</v>
+      </c>
+      <c r="D52" s="33" t="s">
+        <v>96</v>
+      </c>
+      <c r="E52" s="33" t="s">
+        <v>150</v>
       </c>
       <c r="F52" s="8">
         <v>1</v>
@@ -2203,40 +2250,40 @@
       <c r="J52" s="17"/>
       <c r="L52" s="10"/>
     </row>
-    <row r="53" spans="2:12" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="B53" s="18" t="s">
+    <row r="53" spans="2:12" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="B53" s="33" t="s">
         <v>51</v>
       </c>
-      <c r="C53" s="20" t="s">
-        <v>98</v>
-      </c>
-      <c r="D53" s="20" t="s">
-        <v>121</v>
-      </c>
-      <c r="E53" s="20" t="s">
-        <v>152</v>
-      </c>
-      <c r="F53" s="11">
+      <c r="C53" s="34" t="s">
+        <v>97</v>
+      </c>
+      <c r="D53" s="34" t="s">
+        <v>120</v>
+      </c>
+      <c r="E53" s="34" t="s">
+        <v>151</v>
+      </c>
+      <c r="F53" s="38">
         <v>1</v>
       </c>
-      <c r="G53" s="20"/>
+      <c r="G53" s="19"/>
       <c r="H53" s="12"/>
       <c r="I53" s="13"/>
-      <c r="J53" s="33"/>
+      <c r="J53" s="32"/>
       <c r="L53" s="10"/>
     </row>
-    <row r="54" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B54" s="17" t="s">
+    <row r="54" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B54" s="33" t="s">
         <v>52</v>
       </c>
-      <c r="C54" s="17" t="s">
-        <v>99</v>
-      </c>
-      <c r="D54" s="17" t="s">
-        <v>122</v>
-      </c>
-      <c r="E54" s="17" t="s">
-        <v>153</v>
+      <c r="C54" s="33" t="s">
+        <v>98</v>
+      </c>
+      <c r="D54" s="33" t="s">
+        <v>121</v>
+      </c>
+      <c r="E54" s="33" t="s">
+        <v>152</v>
       </c>
       <c r="F54" s="8">
         <v>1</v>
@@ -2247,40 +2294,40 @@
       <c r="J54" s="17"/>
       <c r="L54" s="10"/>
     </row>
-    <row r="55" spans="2:12" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="B55" s="18" t="s">
+    <row r="55" spans="2:12" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="B55" s="33" t="s">
         <v>53</v>
       </c>
-      <c r="C55" s="20" t="s">
-        <v>100</v>
-      </c>
-      <c r="D55" s="20" t="s">
-        <v>123</v>
-      </c>
-      <c r="E55" s="20" t="s">
-        <v>154</v>
+      <c r="C55" s="34" t="s">
+        <v>99</v>
+      </c>
+      <c r="D55" s="34" t="s">
+        <v>122</v>
+      </c>
+      <c r="E55" s="34" t="s">
+        <v>153</v>
       </c>
       <c r="F55" s="11">
         <v>1</v>
       </c>
-      <c r="G55" s="20"/>
+      <c r="G55" s="19"/>
       <c r="H55" s="12"/>
       <c r="I55" s="13"/>
-      <c r="J55" s="33"/>
+      <c r="J55" s="32"/>
       <c r="L55" s="10"/>
     </row>
-    <row r="56" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B56" s="17" t="s">
+    <row r="56" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B56" s="33" t="s">
         <v>54</v>
       </c>
-      <c r="C56" s="17" t="s">
-        <v>101</v>
-      </c>
-      <c r="D56" s="17" t="s">
-        <v>124</v>
-      </c>
-      <c r="E56" s="17" t="s">
-        <v>155</v>
+      <c r="C56" s="33" t="s">
+        <v>100</v>
+      </c>
+      <c r="D56" s="33" t="s">
+        <v>123</v>
+      </c>
+      <c r="E56" s="33" t="s">
+        <v>154</v>
       </c>
       <c r="F56" s="8">
         <v>1</v>
@@ -2291,40 +2338,40 @@
       <c r="J56" s="17"/>
       <c r="L56" s="10"/>
     </row>
-    <row r="57" spans="2:12" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B57" s="18" t="s">
+    <row r="57" spans="2:12" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B57" s="33" t="s">
         <v>55</v>
       </c>
-      <c r="C57" s="20" t="s">
-        <v>102</v>
-      </c>
-      <c r="D57" s="20" t="s">
-        <v>125</v>
-      </c>
-      <c r="E57" s="20" t="s">
-        <v>156</v>
+      <c r="C57" s="34" t="s">
+        <v>101</v>
+      </c>
+      <c r="D57" s="34" t="s">
+        <v>124</v>
+      </c>
+      <c r="E57" s="34" t="s">
+        <v>155</v>
       </c>
       <c r="F57" s="11">
         <v>1</v>
       </c>
-      <c r="G57" s="20"/>
+      <c r="G57" s="19"/>
       <c r="H57" s="12"/>
       <c r="I57" s="13"/>
-      <c r="J57" s="33"/>
+      <c r="J57" s="32"/>
       <c r="L57" s="10"/>
     </row>
-    <row r="58" spans="2:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B58" s="17" t="s">
         <v>56</v>
       </c>
       <c r="C58" s="17" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D58" s="17" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E58" s="17" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="F58" s="8">
         <v>1</v>
@@ -2335,431 +2382,431 @@
       <c r="J58" s="17"/>
       <c r="L58" s="10"/>
     </row>
-    <row r="59" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B59" s="4"/>
-      <c r="C59" s="21"/>
-      <c r="D59" s="21"/>
-      <c r="E59" s="21"/>
+      <c r="C59" s="20"/>
+      <c r="D59" s="20"/>
+      <c r="E59" s="20"/>
       <c r="F59" s="11">
         <f>SUM(F13:F58)</f>
         <v>106</v>
       </c>
-      <c r="G59" s="21"/>
+      <c r="G59" s="20"/>
       <c r="I59" s="14">
         <f>SUM(I13:I58)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="60" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B60" s="4"/>
-      <c r="C60" s="21"/>
-      <c r="D60" s="21"/>
-      <c r="E60" s="21"/>
-      <c r="F60" s="25"/>
-      <c r="G60" s="21"/>
-      <c r="H60" s="27"/>
-      <c r="I60" s="27"/>
-    </row>
-    <row r="61" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="C60" s="20"/>
+      <c r="D60" s="20"/>
+      <c r="E60" s="20"/>
+      <c r="F60" s="24"/>
+      <c r="G60" s="20"/>
+      <c r="H60" s="26"/>
+      <c r="I60" s="26"/>
+    </row>
+    <row r="61" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B61" s="4"/>
-      <c r="C61" s="21"/>
-      <c r="D61" s="21"/>
-      <c r="E61" s="21"/>
-      <c r="F61" s="25"/>
-      <c r="G61" s="21"/>
-      <c r="H61" s="27"/>
-      <c r="I61" s="24"/>
-    </row>
-    <row r="62" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="C61" s="20"/>
+      <c r="D61" s="20"/>
+      <c r="E61" s="20"/>
+      <c r="F61" s="24"/>
+      <c r="G61" s="20"/>
+      <c r="H61" s="26"/>
+      <c r="I61" s="23"/>
+    </row>
+    <row r="62" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B62" s="4"/>
-      <c r="C62" s="21"/>
-      <c r="D62" s="21"/>
-      <c r="E62" s="21"/>
-      <c r="F62" s="25"/>
-      <c r="G62" s="21"/>
-      <c r="H62" s="27"/>
-      <c r="I62" s="24"/>
-    </row>
-    <row r="63" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="C62" s="20"/>
+      <c r="D62" s="20"/>
+      <c r="E62" s="20"/>
+      <c r="F62" s="24"/>
+      <c r="G62" s="20"/>
+      <c r="H62" s="26"/>
+      <c r="I62" s="23"/>
+    </row>
+    <row r="63" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B63" s="4"/>
-      <c r="C63" s="21"/>
-      <c r="D63" s="21"/>
-      <c r="E63" s="21"/>
-      <c r="F63" s="25"/>
-      <c r="G63" s="21"/>
-      <c r="H63" s="25"/>
-      <c r="I63" s="27"/>
+      <c r="C63" s="20"/>
+      <c r="D63" s="20"/>
+      <c r="E63" s="20"/>
+      <c r="F63" s="24"/>
+      <c r="G63" s="20"/>
+      <c r="H63" s="24"/>
+      <c r="I63" s="26"/>
       <c r="J63" s="4"/>
     </row>
-    <row r="64" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="64" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B64" s="4"/>
-      <c r="C64" s="21"/>
-      <c r="D64" s="21"/>
-      <c r="E64" s="21"/>
-      <c r="F64" s="25"/>
-      <c r="G64" s="21"/>
-      <c r="H64" s="25"/>
-      <c r="I64" s="27"/>
+      <c r="C64" s="20"/>
+      <c r="D64" s="20"/>
+      <c r="E64" s="20"/>
+      <c r="F64" s="24"/>
+      <c r="G64" s="20"/>
+      <c r="H64" s="24"/>
+      <c r="I64" s="26"/>
       <c r="J64" s="4"/>
     </row>
-    <row r="65" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="65" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B65" s="4"/>
-      <c r="C65" s="21"/>
-      <c r="D65" s="21"/>
-      <c r="E65" s="21"/>
-      <c r="F65" s="25"/>
-      <c r="G65" s="21"/>
-      <c r="H65" s="25"/>
-      <c r="I65" s="27"/>
+      <c r="C65" s="20"/>
+      <c r="D65" s="20"/>
+      <c r="E65" s="20"/>
+      <c r="F65" s="24"/>
+      <c r="G65" s="20"/>
+      <c r="H65" s="24"/>
+      <c r="I65" s="26"/>
       <c r="J65" s="4"/>
     </row>
-    <row r="66" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="66" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B66" s="4"/>
-      <c r="C66" s="21"/>
-      <c r="D66" s="21"/>
-      <c r="E66" s="21"/>
-      <c r="F66" s="25"/>
-      <c r="G66" s="21"/>
-      <c r="H66" s="25"/>
-      <c r="I66" s="27"/>
+      <c r="C66" s="20"/>
+      <c r="D66" s="20"/>
+      <c r="E66" s="20"/>
+      <c r="F66" s="24"/>
+      <c r="G66" s="20"/>
+      <c r="H66" s="24"/>
+      <c r="I66" s="26"/>
       <c r="J66" s="4"/>
     </row>
-    <row r="67" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="67" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B67" s="4"/>
-      <c r="C67" s="21"/>
-      <c r="D67" s="21"/>
-      <c r="E67" s="21"/>
-      <c r="F67" s="25"/>
-      <c r="G67" s="21"/>
-      <c r="H67" s="25"/>
-      <c r="I67" s="27"/>
+      <c r="C67" s="20"/>
+      <c r="D67" s="20"/>
+      <c r="E67" s="20"/>
+      <c r="F67" s="24"/>
+      <c r="G67" s="20"/>
+      <c r="H67" s="24"/>
+      <c r="I67" s="26"/>
       <c r="J67" s="4"/>
     </row>
-    <row r="68" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="68" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B68" s="4"/>
-      <c r="C68" s="21"/>
-      <c r="D68" s="21"/>
-      <c r="E68" s="21"/>
-      <c r="F68" s="25"/>
-      <c r="G68" s="21"/>
-      <c r="H68" s="25"/>
-      <c r="I68" s="27"/>
+      <c r="C68" s="20"/>
+      <c r="D68" s="20"/>
+      <c r="E68" s="20"/>
+      <c r="F68" s="24"/>
+      <c r="G68" s="20"/>
+      <c r="H68" s="24"/>
+      <c r="I68" s="26"/>
       <c r="J68" s="4"/>
     </row>
-    <row r="69" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="69" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B69" s="4"/>
-      <c r="C69" s="21"/>
-      <c r="D69" s="21"/>
-      <c r="E69" s="21"/>
-      <c r="F69" s="25"/>
-      <c r="G69" s="21"/>
-      <c r="H69" s="25"/>
-      <c r="I69" s="27"/>
+      <c r="C69" s="20"/>
+      <c r="D69" s="20"/>
+      <c r="E69" s="20"/>
+      <c r="F69" s="24"/>
+      <c r="G69" s="20"/>
+      <c r="H69" s="24"/>
+      <c r="I69" s="26"/>
       <c r="J69" s="4"/>
     </row>
-    <row r="70" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="70" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B70" s="4"/>
-      <c r="C70" s="21"/>
-      <c r="D70" s="21"/>
-      <c r="E70" s="21"/>
-      <c r="F70" s="25"/>
-      <c r="G70" s="21"/>
-      <c r="H70" s="25"/>
-      <c r="I70" s="27"/>
+      <c r="C70" s="20"/>
+      <c r="D70" s="20"/>
+      <c r="E70" s="20"/>
+      <c r="F70" s="24"/>
+      <c r="G70" s="20"/>
+      <c r="H70" s="24"/>
+      <c r="I70" s="26"/>
       <c r="J70" s="4"/>
     </row>
-    <row r="71" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="71" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B71" s="4"/>
-      <c r="C71" s="21"/>
-      <c r="D71" s="21"/>
-      <c r="E71" s="21"/>
-      <c r="F71" s="25"/>
-      <c r="G71" s="21"/>
-      <c r="H71" s="25"/>
-      <c r="I71" s="27"/>
+      <c r="C71" s="20"/>
+      <c r="D71" s="20"/>
+      <c r="E71" s="20"/>
+      <c r="F71" s="24"/>
+      <c r="G71" s="20"/>
+      <c r="H71" s="24"/>
+      <c r="I71" s="26"/>
       <c r="J71" s="4"/>
     </row>
-    <row r="72" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="72" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B72" s="4"/>
-      <c r="C72" s="21"/>
-      <c r="D72" s="21"/>
-      <c r="E72" s="21"/>
-      <c r="F72" s="25"/>
-      <c r="G72" s="21"/>
-      <c r="H72" s="25"/>
-      <c r="I72" s="27"/>
+      <c r="C72" s="20"/>
+      <c r="D72" s="20"/>
+      <c r="E72" s="20"/>
+      <c r="F72" s="24"/>
+      <c r="G72" s="20"/>
+      <c r="H72" s="24"/>
+      <c r="I72" s="26"/>
       <c r="J72" s="4"/>
     </row>
-    <row r="73" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="73" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B73" s="4"/>
-      <c r="C73" s="21"/>
-      <c r="D73" s="21"/>
-      <c r="E73" s="21"/>
-      <c r="F73" s="25"/>
-      <c r="G73" s="21"/>
-      <c r="H73" s="25"/>
-      <c r="I73" s="27"/>
+      <c r="C73" s="20"/>
+      <c r="D73" s="20"/>
+      <c r="E73" s="20"/>
+      <c r="F73" s="24"/>
+      <c r="G73" s="20"/>
+      <c r="H73" s="24"/>
+      <c r="I73" s="26"/>
       <c r="J73" s="4"/>
     </row>
-    <row r="74" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="74" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B74" s="4"/>
-      <c r="C74" s="21"/>
-      <c r="D74" s="21"/>
-      <c r="E74" s="21"/>
-      <c r="F74" s="25"/>
-      <c r="G74" s="21"/>
-      <c r="H74" s="25"/>
-      <c r="I74" s="27"/>
+      <c r="C74" s="20"/>
+      <c r="D74" s="20"/>
+      <c r="E74" s="20"/>
+      <c r="F74" s="24"/>
+      <c r="G74" s="20"/>
+      <c r="H74" s="24"/>
+      <c r="I74" s="26"/>
       <c r="J74" s="4"/>
     </row>
-    <row r="75" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="75" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B75" s="4"/>
-      <c r="C75" s="21"/>
-      <c r="D75" s="21"/>
-      <c r="E75" s="21"/>
-      <c r="F75" s="25"/>
-      <c r="G75" s="21"/>
-      <c r="H75" s="25"/>
-      <c r="I75" s="27"/>
+      <c r="C75" s="20"/>
+      <c r="D75" s="20"/>
+      <c r="E75" s="20"/>
+      <c r="F75" s="24"/>
+      <c r="G75" s="20"/>
+      <c r="H75" s="24"/>
+      <c r="I75" s="26"/>
       <c r="J75" s="4"/>
     </row>
-    <row r="76" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="76" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B76" s="4"/>
-      <c r="C76" s="21"/>
-      <c r="D76" s="21"/>
-      <c r="E76" s="21"/>
-      <c r="F76" s="25"/>
-      <c r="G76" s="21"/>
-      <c r="H76" s="25"/>
-      <c r="I76" s="27"/>
+      <c r="C76" s="20"/>
+      <c r="D76" s="20"/>
+      <c r="E76" s="20"/>
+      <c r="F76" s="24"/>
+      <c r="G76" s="20"/>
+      <c r="H76" s="24"/>
+      <c r="I76" s="26"/>
       <c r="J76" s="4"/>
     </row>
-    <row r="77" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="77" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B77" s="4"/>
-      <c r="C77" s="21"/>
-      <c r="D77" s="21"/>
-      <c r="E77" s="21"/>
-      <c r="F77" s="25"/>
-      <c r="G77" s="21"/>
-      <c r="H77" s="25"/>
-      <c r="I77" s="27"/>
+      <c r="C77" s="20"/>
+      <c r="D77" s="20"/>
+      <c r="E77" s="20"/>
+      <c r="F77" s="24"/>
+      <c r="G77" s="20"/>
+      <c r="H77" s="24"/>
+      <c r="I77" s="26"/>
       <c r="J77" s="4"/>
     </row>
-    <row r="78" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="78" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B78" s="4"/>
-      <c r="C78" s="21"/>
-      <c r="D78" s="21"/>
-      <c r="E78" s="21"/>
-      <c r="F78" s="25"/>
-      <c r="G78" s="21"/>
-      <c r="H78" s="25"/>
-      <c r="I78" s="27"/>
+      <c r="C78" s="20"/>
+      <c r="D78" s="20"/>
+      <c r="E78" s="20"/>
+      <c r="F78" s="24"/>
+      <c r="G78" s="20"/>
+      <c r="H78" s="24"/>
+      <c r="I78" s="26"/>
       <c r="J78" s="4"/>
     </row>
-    <row r="79" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="79" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B79" s="4"/>
-      <c r="C79" s="21"/>
-      <c r="D79" s="21"/>
-      <c r="E79" s="21"/>
-      <c r="F79" s="25"/>
-      <c r="G79" s="21"/>
-      <c r="H79" s="25"/>
-      <c r="I79" s="27"/>
+      <c r="C79" s="20"/>
+      <c r="D79" s="20"/>
+      <c r="E79" s="20"/>
+      <c r="F79" s="24"/>
+      <c r="G79" s="20"/>
+      <c r="H79" s="24"/>
+      <c r="I79" s="26"/>
       <c r="J79" s="4"/>
     </row>
-    <row r="80" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="80" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B80" s="4"/>
-      <c r="C80" s="21"/>
-      <c r="D80" s="21"/>
-      <c r="E80" s="21"/>
-      <c r="F80" s="25"/>
-      <c r="G80" s="21"/>
-      <c r="H80" s="25"/>
-      <c r="I80" s="27"/>
+      <c r="C80" s="20"/>
+      <c r="D80" s="20"/>
+      <c r="E80" s="20"/>
+      <c r="F80" s="24"/>
+      <c r="G80" s="20"/>
+      <c r="H80" s="24"/>
+      <c r="I80" s="26"/>
       <c r="J80" s="4"/>
     </row>
-    <row r="81" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="81" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B81" s="4"/>
-      <c r="C81" s="21"/>
-      <c r="D81" s="21"/>
-      <c r="E81" s="21"/>
-      <c r="F81" s="25"/>
-      <c r="G81" s="21"/>
-      <c r="H81" s="25"/>
-      <c r="I81" s="27"/>
+      <c r="C81" s="20"/>
+      <c r="D81" s="20"/>
+      <c r="E81" s="20"/>
+      <c r="F81" s="24"/>
+      <c r="G81" s="20"/>
+      <c r="H81" s="24"/>
+      <c r="I81" s="26"/>
       <c r="J81" s="4"/>
     </row>
-    <row r="82" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="82" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B82" s="4"/>
-      <c r="C82" s="21"/>
-      <c r="D82" s="21"/>
-      <c r="E82" s="21"/>
-      <c r="F82" s="25"/>
-      <c r="G82" s="21"/>
-      <c r="H82" s="25"/>
-      <c r="I82" s="27"/>
+      <c r="C82" s="20"/>
+      <c r="D82" s="20"/>
+      <c r="E82" s="20"/>
+      <c r="F82" s="24"/>
+      <c r="G82" s="20"/>
+      <c r="H82" s="24"/>
+      <c r="I82" s="26"/>
       <c r="J82" s="4"/>
     </row>
-    <row r="83" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="83" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B83" s="4"/>
-      <c r="C83" s="21"/>
-      <c r="D83" s="21"/>
-      <c r="E83" s="21"/>
-      <c r="F83" s="25"/>
-      <c r="G83" s="21"/>
-      <c r="H83" s="25"/>
-      <c r="I83" s="27"/>
+      <c r="C83" s="20"/>
+      <c r="D83" s="20"/>
+      <c r="E83" s="20"/>
+      <c r="F83" s="24"/>
+      <c r="G83" s="20"/>
+      <c r="H83" s="24"/>
+      <c r="I83" s="26"/>
       <c r="J83" s="4"/>
     </row>
-    <row r="84" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="84" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B84" s="4"/>
-      <c r="C84" s="21"/>
-      <c r="D84" s="21"/>
-      <c r="E84" s="21"/>
-      <c r="F84" s="25"/>
-      <c r="G84" s="21"/>
-      <c r="H84" s="25"/>
-      <c r="I84" s="27"/>
+      <c r="C84" s="20"/>
+      <c r="D84" s="20"/>
+      <c r="E84" s="20"/>
+      <c r="F84" s="24"/>
+      <c r="G84" s="20"/>
+      <c r="H84" s="24"/>
+      <c r="I84" s="26"/>
       <c r="J84" s="4"/>
     </row>
-    <row r="85" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="85" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B85" s="4"/>
-      <c r="C85" s="21"/>
-      <c r="D85" s="21"/>
-      <c r="E85" s="21"/>
-      <c r="F85" s="25"/>
-      <c r="G85" s="21"/>
-      <c r="H85" s="25"/>
-      <c r="I85" s="27"/>
+      <c r="C85" s="20"/>
+      <c r="D85" s="20"/>
+      <c r="E85" s="20"/>
+      <c r="F85" s="24"/>
+      <c r="G85" s="20"/>
+      <c r="H85" s="24"/>
+      <c r="I85" s="26"/>
       <c r="J85" s="4"/>
     </row>
-    <row r="86" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="86" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B86" s="4"/>
-      <c r="C86" s="21"/>
-      <c r="D86" s="21"/>
-      <c r="E86" s="21"/>
-      <c r="F86" s="25"/>
-      <c r="G86" s="21"/>
-      <c r="H86" s="25"/>
-      <c r="I86" s="27"/>
+      <c r="C86" s="20"/>
+      <c r="D86" s="20"/>
+      <c r="E86" s="20"/>
+      <c r="F86" s="24"/>
+      <c r="G86" s="20"/>
+      <c r="H86" s="24"/>
+      <c r="I86" s="26"/>
       <c r="J86" s="4"/>
     </row>
-    <row r="87" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="87" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B87" s="4"/>
-      <c r="C87" s="21"/>
-      <c r="D87" s="21"/>
-      <c r="E87" s="21"/>
-      <c r="F87" s="25"/>
-      <c r="G87" s="21"/>
-      <c r="H87" s="25"/>
-      <c r="I87" s="27"/>
+      <c r="C87" s="20"/>
+      <c r="D87" s="20"/>
+      <c r="E87" s="20"/>
+      <c r="F87" s="24"/>
+      <c r="G87" s="20"/>
+      <c r="H87" s="24"/>
+      <c r="I87" s="26"/>
       <c r="J87" s="4"/>
     </row>
-    <row r="88" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="88" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B88" s="4"/>
-      <c r="C88" s="21"/>
-      <c r="D88" s="21"/>
-      <c r="E88" s="21"/>
-      <c r="F88" s="25"/>
-      <c r="G88" s="21"/>
-      <c r="H88" s="25"/>
-      <c r="I88" s="27"/>
+      <c r="C88" s="20"/>
+      <c r="D88" s="20"/>
+      <c r="E88" s="20"/>
+      <c r="F88" s="24"/>
+      <c r="G88" s="20"/>
+      <c r="H88" s="24"/>
+      <c r="I88" s="26"/>
       <c r="J88" s="4"/>
     </row>
-    <row r="89" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="89" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B89" s="4"/>
-      <c r="C89" s="21"/>
-      <c r="D89" s="21"/>
-      <c r="E89" s="21"/>
-      <c r="F89" s="25"/>
-      <c r="G89" s="21"/>
-      <c r="H89" s="25"/>
-      <c r="I89" s="27"/>
+      <c r="C89" s="20"/>
+      <c r="D89" s="20"/>
+      <c r="E89" s="20"/>
+      <c r="F89" s="24"/>
+      <c r="G89" s="20"/>
+      <c r="H89" s="24"/>
+      <c r="I89" s="26"/>
       <c r="J89" s="4"/>
     </row>
-    <row r="90" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="90" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B90" s="4"/>
-      <c r="C90" s="21"/>
-      <c r="D90" s="21"/>
-      <c r="E90" s="21"/>
-      <c r="F90" s="25"/>
-      <c r="G90" s="21"/>
-      <c r="H90" s="25"/>
-      <c r="I90" s="27"/>
+      <c r="C90" s="20"/>
+      <c r="D90" s="20"/>
+      <c r="E90" s="20"/>
+      <c r="F90" s="24"/>
+      <c r="G90" s="20"/>
+      <c r="H90" s="24"/>
+      <c r="I90" s="26"/>
       <c r="J90" s="4"/>
     </row>
-    <row r="91" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="E91" s="22"/>
-      <c r="F91" s="26"/>
-      <c r="G91" s="22"/>
-      <c r="H91" s="26"/>
-      <c r="I91" s="28"/>
-      <c r="J91" s="22"/>
-    </row>
-    <row r="93" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="91" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="E91" s="21"/>
+      <c r="F91" s="25"/>
+      <c r="G91" s="21"/>
+      <c r="H91" s="25"/>
+      <c r="I91" s="27"/>
+      <c r="J91" s="21"/>
+    </row>
+    <row r="93" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B93" s="4"/>
       <c r="C93" s="4"/>
       <c r="D93" s="4"/>
       <c r="E93" s="4"/>
-      <c r="F93" s="24"/>
+      <c r="F93" s="23"/>
       <c r="G93" s="4"/>
-      <c r="H93" s="24"/>
-      <c r="I93" s="24"/>
+      <c r="H93" s="23"/>
+      <c r="I93" s="23"/>
       <c r="J93" s="4"/>
     </row>
-    <row r="94" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="94" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B94" s="4"/>
       <c r="C94" s="4"/>
       <c r="D94" s="4"/>
       <c r="E94" s="4"/>
-      <c r="F94" s="24"/>
+      <c r="F94" s="23"/>
       <c r="G94" s="4"/>
-      <c r="H94" s="24"/>
-      <c r="I94" s="24"/>
+      <c r="H94" s="23"/>
+      <c r="I94" s="23"/>
       <c r="J94" s="4"/>
     </row>
-    <row r="95" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="95" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B95" s="4"/>
       <c r="C95" s="4"/>
       <c r="D95" s="4"/>
       <c r="E95" s="4"/>
-      <c r="F95" s="24"/>
+      <c r="F95" s="23"/>
       <c r="G95" s="4"/>
-      <c r="H95" s="24"/>
-      <c r="I95" s="24"/>
+      <c r="H95" s="23"/>
+      <c r="I95" s="23"/>
       <c r="J95" s="4"/>
     </row>
-    <row r="96" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="96" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B96" s="4"/>
       <c r="C96" s="4"/>
       <c r="D96" s="4"/>
       <c r="E96" s="4"/>
-      <c r="F96" s="24"/>
+      <c r="F96" s="23"/>
       <c r="G96" s="4"/>
-      <c r="H96" s="24"/>
-      <c r="I96" s="24"/>
+      <c r="H96" s="23"/>
+      <c r="I96" s="23"/>
       <c r="J96" s="4"/>
     </row>
-    <row r="97" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="97" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B97" s="4"/>
       <c r="C97" s="4"/>
       <c r="D97" s="4"/>
       <c r="E97" s="4"/>
-      <c r="F97" s="24"/>
+      <c r="F97" s="23"/>
       <c r="G97" s="4"/>
-      <c r="H97" s="24"/>
-      <c r="I97" s="24"/>
+      <c r="H97" s="23"/>
+      <c r="I97" s="23"/>
       <c r="J97" s="4"/>
     </row>
-    <row r="98" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="98" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B98" s="4"/>
       <c r="C98" s="4"/>
       <c r="D98" s="4"/>
       <c r="E98" s="4"/>
-      <c r="F98" s="24"/>
+      <c r="F98" s="23"/>
       <c r="G98" s="4"/>
-      <c r="H98" s="24"/>
-      <c r="I98" s="24"/>
+      <c r="H98" s="23"/>
+      <c r="I98" s="23"/>
       <c r="J98" s="4"/>
     </row>
   </sheetData>
@@ -2772,7 +2819,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2781,7 +2828,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>